<commit_message>
fix(examples): Blatt/Spalten-Verweise von FB-01 passen zur Zeichnung
24 von 40 Verweisen in Stueckliste und Klemmenplan zeigten auf falsche Spalten
(z. B. -M1 /3.8, gezeichnet in Spalte 5). Die Zeichnung bleibt, die Verweise in
scripts/example_docs/data.py und make_rest.py folgen ihr; Dokumente neu erzeugt.

- test_example_consistency: jeder Verweis zeigt auf die Spalte, in der das
  Kennzeichen im PDF steht (53 Faelle)
- .gitattributes: PDF/XLSX/PNG binaer, core.autocrlf veraendert sie nicht mehr
- load_example.py --refresh laedt die Beispieldokumente neu hoch

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/foerderband/02_Stueckliste_FB-01.xlsx
+++ b/examples/foerderband/02_Stueckliste_FB-01.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stueckliste" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Stueckliste" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -510,7 +510,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>/2.1</t>
+          <t>/2.2</t>
         </is>
       </c>
     </row>
@@ -690,7 +690,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>/4.3</t>
+          <t>/4.2</t>
         </is>
       </c>
     </row>
@@ -720,7 +720,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>/3.8</t>
+          <t>/3.5</t>
         </is>
       </c>
     </row>
@@ -840,7 +840,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>/5.4</t>
+          <t>/5.5</t>
         </is>
       </c>
     </row>
@@ -930,7 +930,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>/6.6</t>
+          <t>/6.5</t>
         </is>
       </c>
     </row>
@@ -1140,7 +1140,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>/3.8</t>
+          <t>/3.5</t>
         </is>
       </c>
     </row>
@@ -1200,7 +1200,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>/5.4</t>
+          <t>/5.5</t>
         </is>
       </c>
     </row>
@@ -1260,7 +1260,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>/3.8</t>
+          <t>/3.5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(examples): Beispielanlage FB-01 mit fuenf Einbauorten und vier weiteren Betriebsmitteln
contract.md Abschnitt 5 verlangt >= 5 Baugruppen und >= 20 Teile; FB-01 hatte nur +ST1 und +FE1 mit 18 Teilen. Neue Einbauorte +BP1 Bedienpult, +AN1 Antrieb, +SE1 Einlauf, +SA1 Auslauf (statt +FE1) und die Geraete -F3, -Q2, -H3, -P1 ohne Aenderung an SPS-Programm und E/A-Belegung, damit die Eval-Fragen gelten. Alles aus data.py erzeugt; Konsistenztest prueft jeden Blattverweis, neue Tests rechnen das Modell aus der Stueckliste nach (5 Zonen, 22 Teile).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/foerderband/02_Stueckliste_FB-01.xlsx
+++ b/examples/foerderband/02_Stueckliste_FB-01.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Stueckliste" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stueckliste" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -443,7 +443,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Anlage =FB1, Schaltschrank +ST1, Feld +FE1. Beispielanlage, frei erfunden, ohne Herstellerbezug.</t>
+          <t>Anlage =FB1: Schaltschrank +ST1, Bedienpult +BP1, Antrieb +AN1, Einlauf +SE1, Auslauf +SA1. Beispielanlage, frei erfunden, ohne Herstellerbezug.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -577,17 +577,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>-T1</t>
+          <t>-F3</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Netzteil 230 V AC / 24 V DC, 5 A</t>
+          <t>Leitungsschutzschalter 24 V Steuerkreis Bedienpult</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Schaltnetzteil 24V/5A</t>
+          <t>LS-Schalter 1P B4 (DC)</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -607,17 +607,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>-K1</t>
+          <t>-T1</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Schuetz Foerdermotor vorwaerts</t>
+          <t>Netzteil 230 V AC / 24 V DC, 5 A</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Leistungsschuetz 4 kW, Spule 24 V DC</t>
+          <t>Schaltnetzteil 24V/5A</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -630,19 +630,19 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>/3.4</t>
+          <t>/2.6</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>-K2</t>
+          <t>-K1</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Schuetz Foerdermotor rueckwaerts</t>
+          <t>Schuetz Foerdermotor vorwaerts</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -660,24 +660,24 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>/3.6</t>
+          <t>/3.4</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>-K3</t>
+          <t>-K2</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Sicherheitsrelais Not-Halt, 2-kanalig</t>
+          <t>Schuetz Foerdermotor rueckwaerts</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Sicherheitsschaltgeraet Kat. 3 / PL d</t>
+          <t>Leistungsschuetz 4 kW, Spule 24 V DC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -690,24 +690,24 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>/4.2</t>
+          <t>/3.6</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>-M1</t>
+          <t>-K3</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Foerdermotor 3~ 1,5 kW, 1420 1/min</t>
+          <t>Sicherheitsrelais Not-Halt, 2-kanalig</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Drehstrommotor 1,5 kW, IE3</t>
+          <t>Sicherheitsschaltgeraet Kat. 3 / PL d</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -715,29 +715,29 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>+FE1</t>
+          <t>+ST1</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>/3.5</t>
+          <t>/4.2</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>-S1</t>
+          <t>-M1</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Taster Start (Schliesser)</t>
+          <t>Foerdermotor 3~ 1,5 kW, 1420 1/min</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Drucktaster gruen 1S</t>
+          <t>Drehstrommotor 1,5 kW, IE3</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -745,29 +745,29 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>+FE1</t>
+          <t>+AN1</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>/4.6</t>
+          <t>/3.5</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>-S2</t>
+          <t>-Q2</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Taster Stop (Oeffner)</t>
+          <t>Reparaturschalter Foerdermotor, 3-polig, abschliessbar</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Drucktaster rot 1OE</t>
+          <t>Lasttrennschalter 3P 16A im Gehaeuse</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -775,29 +775,29 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>+FE1</t>
+          <t>+AN1</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>/4.7</t>
+          <t>/3.5</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>-S3</t>
+          <t>-S1</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Not-Halt-Taster, 2 Oeffner, rastend</t>
+          <t>Taster Start (Schliesser)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Pilzdrucktaster 2OE</t>
+          <t>Drucktaster gruen 1S</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -805,29 +805,29 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>+FE1</t>
+          <t>+BP1</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>/4.2</t>
+          <t>/4.6</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>-B1</t>
+          <t>-S2</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Lichtschranke Einlauf</t>
+          <t>Taster Stop (Oeffner)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Reflexionslichtschranke 24 V DC PNP</t>
+          <t>Drucktaster rot 1OE</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -835,29 +835,29 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>+FE1</t>
+          <t>+BP1</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>/5.5</t>
+          <t>/4.7</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>-B2</t>
+          <t>-S3</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Lichtschranke Auslauf</t>
+          <t>Not-Halt-Taster, 2 Oeffner, rastend</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Reflexionslichtschranke 24 V DC PNP</t>
+          <t>Pilzdrucktaster 2OE</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -865,29 +865,29 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>+FE1</t>
+          <t>+BP1</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>/5.5</t>
+          <t>/4.2</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>-H1</t>
+          <t>-B1</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Meldeleuchte Betrieb (gruen)</t>
+          <t>Lichtschranke Einlauf</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>LED-Leuchtmelder 24 V DC gruen</t>
+          <t>Reflexionslichtschranke 24 V DC PNP</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -895,29 +895,29 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>+FE1</t>
+          <t>+SE1</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>/6.5</t>
+          <t>/5.5</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>-H2</t>
+          <t>-B2</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Meldeleuchte Stoerung (rot)</t>
+          <t>Lichtschranke Auslauf</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>LED-Leuchtmelder 24 V DC rot</t>
+          <t>Reflexionslichtschranke 24 V DC PNP</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -925,29 +925,29 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>+FE1</t>
+          <t>+SA1</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>/6.5</t>
+          <t>/5.5</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>-A1</t>
+          <t>-H1</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>SPS CPU, kompakt, PROFIBUS DP</t>
+          <t>Meldeleuchte Betrieb (gruen)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>SPS-Zentralbaugruppe</t>
+          <t>LED-Leuchtmelder 24 V DC gruen</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -955,29 +955,29 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>+ST1</t>
+          <t>+BP1</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>/5.1</t>
+          <t>/6.5</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>-A1.1</t>
+          <t>-H2</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Digitaleingabe 16 x 24 V DC</t>
+          <t>Meldeleuchte Stoerung (rot)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>DI-Baugruppe 16 DI</t>
+          <t>LED-Leuchtmelder 24 V DC rot</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -985,29 +985,29 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>+ST1</t>
+          <t>+BP1</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>/5.2</t>
+          <t>/6.5</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>-A1.2</t>
+          <t>-H3</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Digitalausgabe 16 x 24 V DC / 0,5 A</t>
+          <t>Meldeleuchte Not-Halt betaetigt (gelb)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>DO-Baugruppe 16 DO</t>
+          <t>LED-Leuchtmelder 24 V DC gelb</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -1015,63 +1015,63 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>+ST1</t>
+          <t>+BP1</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>/6.2</t>
+          <t>/4.8</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>-X1</t>
+          <t>-P1</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Klemmleiste Netzeinspeisung</t>
+          <t>Betriebsstundenzaehler Foerderband</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Reihenklemme 4 mm2</t>
+          <t>Betriebsstundenzaehler 24 V DC, 7-stellig</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>+ST1</t>
+          <t>+BP1</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>/2.1</t>
+          <t>/6.6</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>-X2</t>
+          <t>-A1</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Klemmleiste 24 V Steuerspannung</t>
+          <t>SPS CPU, kompakt, PROFIBUS DP</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Reihenklemme 2,5 mm2</t>
+          <t>SPS-Zentralbaugruppe</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1080,28 +1080,28 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>/2.7</t>
+          <t>/5.1</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>-X3</t>
+          <t>-A1.1</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Klemmleiste Feldgeraete (Sensoren, Taster)</t>
+          <t>Digitaleingabe 16 x 24 V DC</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Reihenklemme 2,5 mm2</t>
+          <t>DI-Baugruppe 16 DI</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1110,155 +1110,275 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>/5.3</t>
+          <t>/5.2</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>-X4</t>
+          <t>-A1.2</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Klemmleiste Motorabgang</t>
+          <t>Digitalausgabe 16 x 24 V DC / 0,5 A</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
+          <t>DO-Baugruppe 16 DO</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>+ST1</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>/6.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>-X1</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Klemmleiste Netzeinspeisung</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
           <t>Reihenklemme 4 mm2</t>
         </is>
       </c>
-      <c r="D26" t="n">
-        <v>4</v>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>+ST1</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>/3.5</t>
+      <c r="D27" t="n">
+        <v>5</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>+ST1</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>/2.1</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>-W1</t>
+          <t>-X2</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Steuerleitung Bedienpult</t>
+          <t>Klemmleiste 24 V Steuerspannung</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>12 x 0,75 mm2, 8 m</t>
+          <t>Reihenklemme 2,5 mm2</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>+ST1 -&gt; +FE1</t>
+          <t>+ST1</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>/4.6</t>
+          <t>/2.7</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>-W2</t>
+          <t>-X3</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Sensorleitung Lichtschranke Einlauf</t>
+          <t>Klemmleiste Feldgeraete (Sensoren, Taster, Leuchten)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>4 x 0,5 mm2, 6 m</t>
+          <t>Reihenklemme 2,5 mm2</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>+ST1 -&gt; +FE1</t>
+          <t>+ST1</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>/5.5</t>
+          <t>/5.3</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>-X4</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Klemmleiste Motorabgang</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Reihenklemme 4 mm2</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>4</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>+ST1</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>/3.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>-W1</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Steuerleitung Bedienpult</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>12 x 0,75 mm2, 8 m</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>+ST1 -&gt; +BP1</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>/4.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>-W2</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Sensorleitung Lichtschranke Einlauf</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>4 x 0,5 mm2, 6 m</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>+ST1 -&gt; +SE1</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>/5.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t>-W3</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>Sensorleitung Lichtschranke Auslauf</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>4 x 0,5 mm2, 9 m</t>
         </is>
       </c>
-      <c r="D30" t="n">
-        <v>1</v>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>+ST1 -&gt; +FE1</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
+      <c r="D34" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>+ST1 -&gt; +SA1</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
         <is>
           <t>/5.5</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
+    <row r="35">
+      <c r="A35" t="inlineStr">
         <is>
           <t>-W4</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>Motorleitung</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>4G2,5 mm2, 7 m</t>
         </is>
       </c>
-      <c r="D31" t="n">
-        <v>1</v>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>+ST1 -&gt; +FE1</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
+      <c r="D35" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>+ST1 -&gt; +AN1</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
         <is>
           <t>/3.5</t>
         </is>

</xml_diff>

<commit_message>
feat(examples): Beispielanlage FB-01 mit fünf Einbauorten und 22 Teilen (Kriterium 2) (#42)
* feat(examples): Beispielanlage FB-01 mit fuenf Einbauorten und vier weiteren Betriebsmitteln

contract.md Abschnitt 5 verlangt >= 5 Baugruppen und >= 20 Teile; FB-01 hatte nur +ST1 und +FE1 mit 18 Teilen. Neue Einbauorte +BP1 Bedienpult, +AN1 Antrieb, +SE1 Einlauf, +SA1 Auslauf (statt +FE1) und die Geraete -F3, -Q2, -H3, -P1 ohne Aenderung an SPS-Programm und E/A-Belegung, damit die Eval-Fragen gelten. Alles aus data.py erzeugt; Konsistenztest prueft jeden Blattverweis, neue Tests rechnen das Modell aus der Stueckliste nach (5 Zonen, 22 Teile).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>

* docs(product): Kriterium 2 mit erweiterter Beispielanlage, Beispielcodes in README und AGENTS

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>

---------

Co-authored-by: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/foerderband/02_Stueckliste_FB-01.xlsx
+++ b/examples/foerderband/02_Stueckliste_FB-01.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Stueckliste" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stueckliste" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -443,7 +443,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Anlage =FB1, Schaltschrank +ST1, Feld +FE1. Beispielanlage, frei erfunden, ohne Herstellerbezug.</t>
+          <t>Anlage =FB1: Schaltschrank +ST1, Bedienpult +BP1, Antrieb +AN1, Einlauf +SE1, Auslauf +SA1. Beispielanlage, frei erfunden, ohne Herstellerbezug.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -577,17 +577,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>-T1</t>
+          <t>-F3</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Netzteil 230 V AC / 24 V DC, 5 A</t>
+          <t>Leitungsschutzschalter 24 V Steuerkreis Bedienpult</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Schaltnetzteil 24V/5A</t>
+          <t>LS-Schalter 1P B4 (DC)</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -607,17 +607,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>-K1</t>
+          <t>-T1</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Schuetz Foerdermotor vorwaerts</t>
+          <t>Netzteil 230 V AC / 24 V DC, 5 A</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Leistungsschuetz 4 kW, Spule 24 V DC</t>
+          <t>Schaltnetzteil 24V/5A</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -630,19 +630,19 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>/3.4</t>
+          <t>/2.6</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>-K2</t>
+          <t>-K1</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Schuetz Foerdermotor rueckwaerts</t>
+          <t>Schuetz Foerdermotor vorwaerts</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -660,24 +660,24 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>/3.6</t>
+          <t>/3.4</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>-K3</t>
+          <t>-K2</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Sicherheitsrelais Not-Halt, 2-kanalig</t>
+          <t>Schuetz Foerdermotor rueckwaerts</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Sicherheitsschaltgeraet Kat. 3 / PL d</t>
+          <t>Leistungsschuetz 4 kW, Spule 24 V DC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -690,24 +690,24 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>/4.2</t>
+          <t>/3.6</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>-M1</t>
+          <t>-K3</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Foerdermotor 3~ 1,5 kW, 1420 1/min</t>
+          <t>Sicherheitsrelais Not-Halt, 2-kanalig</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Drehstrommotor 1,5 kW, IE3</t>
+          <t>Sicherheitsschaltgeraet Kat. 3 / PL d</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -715,29 +715,29 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>+FE1</t>
+          <t>+ST1</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>/3.5</t>
+          <t>/4.2</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>-S1</t>
+          <t>-M1</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Taster Start (Schliesser)</t>
+          <t>Foerdermotor 3~ 1,5 kW, 1420 1/min</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Drucktaster gruen 1S</t>
+          <t>Drehstrommotor 1,5 kW, IE3</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -745,29 +745,29 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>+FE1</t>
+          <t>+AN1</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>/4.6</t>
+          <t>/3.5</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>-S2</t>
+          <t>-Q2</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Taster Stop (Oeffner)</t>
+          <t>Reparaturschalter Foerdermotor, 3-polig, abschliessbar</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Drucktaster rot 1OE</t>
+          <t>Lasttrennschalter 3P 16A im Gehaeuse</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -775,29 +775,29 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>+FE1</t>
+          <t>+AN1</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>/4.7</t>
+          <t>/3.5</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>-S3</t>
+          <t>-S1</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Not-Halt-Taster, 2 Oeffner, rastend</t>
+          <t>Taster Start (Schliesser)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Pilzdrucktaster 2OE</t>
+          <t>Drucktaster gruen 1S</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -805,29 +805,29 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>+FE1</t>
+          <t>+BP1</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>/4.2</t>
+          <t>/4.6</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>-B1</t>
+          <t>-S2</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Lichtschranke Einlauf</t>
+          <t>Taster Stop (Oeffner)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Reflexionslichtschranke 24 V DC PNP</t>
+          <t>Drucktaster rot 1OE</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -835,29 +835,29 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>+FE1</t>
+          <t>+BP1</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>/5.5</t>
+          <t>/4.7</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>-B2</t>
+          <t>-S3</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Lichtschranke Auslauf</t>
+          <t>Not-Halt-Taster, 2 Oeffner, rastend</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Reflexionslichtschranke 24 V DC PNP</t>
+          <t>Pilzdrucktaster 2OE</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -865,29 +865,29 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>+FE1</t>
+          <t>+BP1</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>/5.5</t>
+          <t>/4.2</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>-H1</t>
+          <t>-B1</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Meldeleuchte Betrieb (gruen)</t>
+          <t>Lichtschranke Einlauf</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>LED-Leuchtmelder 24 V DC gruen</t>
+          <t>Reflexionslichtschranke 24 V DC PNP</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -895,29 +895,29 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>+FE1</t>
+          <t>+SE1</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>/6.5</t>
+          <t>/5.5</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>-H2</t>
+          <t>-B2</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Meldeleuchte Stoerung (rot)</t>
+          <t>Lichtschranke Auslauf</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>LED-Leuchtmelder 24 V DC rot</t>
+          <t>Reflexionslichtschranke 24 V DC PNP</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -925,29 +925,29 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>+FE1</t>
+          <t>+SA1</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>/6.5</t>
+          <t>/5.5</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>-A1</t>
+          <t>-H1</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>SPS CPU, kompakt, PROFIBUS DP</t>
+          <t>Meldeleuchte Betrieb (gruen)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>SPS-Zentralbaugruppe</t>
+          <t>LED-Leuchtmelder 24 V DC gruen</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -955,29 +955,29 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>+ST1</t>
+          <t>+BP1</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>/5.1</t>
+          <t>/6.5</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>-A1.1</t>
+          <t>-H2</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Digitaleingabe 16 x 24 V DC</t>
+          <t>Meldeleuchte Stoerung (rot)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>DI-Baugruppe 16 DI</t>
+          <t>LED-Leuchtmelder 24 V DC rot</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -985,29 +985,29 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>+ST1</t>
+          <t>+BP1</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>/5.2</t>
+          <t>/6.5</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>-A1.2</t>
+          <t>-H3</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Digitalausgabe 16 x 24 V DC / 0,5 A</t>
+          <t>Meldeleuchte Not-Halt betaetigt (gelb)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>DO-Baugruppe 16 DO</t>
+          <t>LED-Leuchtmelder 24 V DC gelb</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -1015,63 +1015,63 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>+ST1</t>
+          <t>+BP1</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>/6.2</t>
+          <t>/4.8</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>-X1</t>
+          <t>-P1</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Klemmleiste Netzeinspeisung</t>
+          <t>Betriebsstundenzaehler Foerderband</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Reihenklemme 4 mm2</t>
+          <t>Betriebsstundenzaehler 24 V DC, 7-stellig</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>+ST1</t>
+          <t>+BP1</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>/2.1</t>
+          <t>/6.6</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>-X2</t>
+          <t>-A1</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Klemmleiste 24 V Steuerspannung</t>
+          <t>SPS CPU, kompakt, PROFIBUS DP</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Reihenklemme 2,5 mm2</t>
+          <t>SPS-Zentralbaugruppe</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1080,28 +1080,28 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>/2.7</t>
+          <t>/5.1</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>-X3</t>
+          <t>-A1.1</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Klemmleiste Feldgeraete (Sensoren, Taster)</t>
+          <t>Digitaleingabe 16 x 24 V DC</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Reihenklemme 2,5 mm2</t>
+          <t>DI-Baugruppe 16 DI</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1110,155 +1110,275 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>/5.3</t>
+          <t>/5.2</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>-X4</t>
+          <t>-A1.2</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Klemmleiste Motorabgang</t>
+          <t>Digitalausgabe 16 x 24 V DC / 0,5 A</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
+          <t>DO-Baugruppe 16 DO</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>+ST1</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>/6.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>-X1</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Klemmleiste Netzeinspeisung</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
           <t>Reihenklemme 4 mm2</t>
         </is>
       </c>
-      <c r="D26" t="n">
-        <v>4</v>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>+ST1</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>/3.5</t>
+      <c r="D27" t="n">
+        <v>5</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>+ST1</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>/2.1</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>-W1</t>
+          <t>-X2</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Steuerleitung Bedienpult</t>
+          <t>Klemmleiste 24 V Steuerspannung</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>12 x 0,75 mm2, 8 m</t>
+          <t>Reihenklemme 2,5 mm2</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>+ST1 -&gt; +FE1</t>
+          <t>+ST1</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>/4.6</t>
+          <t>/2.7</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>-W2</t>
+          <t>-X3</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Sensorleitung Lichtschranke Einlauf</t>
+          <t>Klemmleiste Feldgeraete (Sensoren, Taster, Leuchten)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>4 x 0,5 mm2, 6 m</t>
+          <t>Reihenklemme 2,5 mm2</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>+ST1 -&gt; +FE1</t>
+          <t>+ST1</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>/5.5</t>
+          <t>/5.3</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>-X4</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Klemmleiste Motorabgang</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Reihenklemme 4 mm2</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>4</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>+ST1</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>/3.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>-W1</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Steuerleitung Bedienpult</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>12 x 0,75 mm2, 8 m</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>+ST1 -&gt; +BP1</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>/4.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>-W2</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Sensorleitung Lichtschranke Einlauf</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>4 x 0,5 mm2, 6 m</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>+ST1 -&gt; +SE1</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>/5.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t>-W3</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>Sensorleitung Lichtschranke Auslauf</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>4 x 0,5 mm2, 9 m</t>
         </is>
       </c>
-      <c r="D30" t="n">
-        <v>1</v>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>+ST1 -&gt; +FE1</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
+      <c r="D34" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>+ST1 -&gt; +SA1</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
         <is>
           <t>/5.5</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
+    <row r="35">
+      <c r="A35" t="inlineStr">
         <is>
           <t>-W4</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>Motorleitung</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>4G2,5 mm2, 7 m</t>
         </is>
       </c>
-      <c r="D31" t="n">
-        <v>1</v>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>+ST1 -&gt; +FE1</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
+      <c r="D35" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>+ST1 -&gt; +AN1</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
         <is>
           <t>/3.5</t>
         </is>

</xml_diff>